<commit_message>
chore: 自动同步公告/奖励 0.1.7.2 @ 2026-09-11 12:57
</commit_message>
<xml_diff>
--- a/DT_公告数据表.xlsx
+++ b/DT_公告数据表.xlsx
@@ -67,32 +67,36 @@
     <t xml:space="preserve">详情韩文</t>
   </si>
   <si>
-    <t xml:space="preserve">Version:V 0.1.6.3
-1.Enhance skill damage range;
-2.Make resources easier to obtain;
-3.Improve ad response speed;
-4.Fix several bugs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">版本号:V 0.1.6.3
+    <t xml:space="preserve">Version: V 0.1.6.4
+1. Enhanced skill damage range;  
+2. Easier resource acquisition;  
+3. Improved ad response speed;  
+4. Fixed the issue where watching ads during combat caused game crashes;  
+5. Resolved several bugs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">版本号:V 0.1.6.4
 1.增强技能伤害范围；
 2.资源获得更容易；
-3.提升广告响应速度：
-4.修复若干Bug。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">バージョン:V 0.1.6.3
+3.提升广告响应速度;
+4.修复战斗中观看广告，导致游戏卡死的问题;
+5.修复若干Bug。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">バージョン:V 0.1.6.4
 1.スキルのダメージ範囲を強化；
 2.リソースの獲得を容易に；
 3.広告の応答速度を向上；
-4.いくつかのバグを修正。</t>
-  </si>
-  <si>
-    <t xml:space="preserve">버전:V 0.1.6.3
+4.戦闘中に広告を視聴するとゲームがフリーズする問題を修正；
+5.いくつかのバグを修正。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">버전:V 0.1.6.4
 1.스킬 피해 범위 강화；
 2.자원 획득 용이；
 3.광고 응답 속도 향상；
-4.여러 버그 수정。</t>
+4.전투 중 광고 시청으로 게임이 멈추는 문제 수정；
+5.여러 버그 수정。</t>
   </si>
 </sst>
 </file>
@@ -156,15 +160,12 @@
   <cellStyleXfs count="1">
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf applyAlignment="false" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,11 +487,11 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="5.802816901408451"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="2" min="2" style="0" width="58.08450704225352"/>
     <col collapsed="false" customWidth="true" hidden="false" max="3" min="3" style="0" width="40.394366197183096"/>
     <col collapsed="false" customWidth="true" hidden="false" max="4" min="4" style="0" width="42.647887323943664"/>
     <col collapsed="false" customWidth="true" hidden="false" max="5" min="5" style="0" width="50.42253521126761"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="5.802816901408451"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="2" min="2" style="0" width="58.08450704225352"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,16 +515,16 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>